<commit_message>
Add Basis Menge, Stellplätze, Lademeter, Volumen columns to all 4 reports
Expanded all customer report scripts from 25 to 29 columns:
- Col 12 Basis Menge: billing dimension value (billing_kg or stpl)
- Col 16 Stellplätze: raw value from source data
- Col 17 Lademeter: raw value from source data
- Col 18 Volumen: raw value from source data

Updated EUR_COLS, NUM_RIGHT (right-align), widths in Helu, Sika, SSC, GEZE.

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/geze_dinas_vergleich.xlsx
+++ b/output/billing_report/geze_dinas_vergleich.xlsx
@@ -120,10 +120,10 @@
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -132,10 +132,10 @@
     <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y29"/>
+  <dimension ref="A1:AC29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -517,20 +517,24 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
     <col width="9" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
     <col width="9" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="9" customWidth="1" min="25" max="25"/>
+    <col width="9" customWidth="1" min="26" max="26"/>
+    <col width="9" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -598,70 +602,90 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
+          <t>Basis Menge</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
           <t>Basispreis</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Eff. Preis</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Tonnage kg</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Stellplätze</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Lademeter</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Volumen</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Soll EUR</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Fracht EUR</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Diesel EUR</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Maut EUR</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>Lademittel</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Peak EUR</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Neben EUR</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>EUST Zoll</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Versich.</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Erlöse</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>Abw. Grund</t>
         </is>
@@ -729,45 +753,55 @@
         </is>
       </c>
       <c r="L4" s="6" t="n">
+        <v>8200</v>
+      </c>
+      <c r="M4" s="7" t="n">
         <v>26.41999999999999</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="N4" s="7" t="n">
         <v>28.48399803052683</v>
       </c>
-      <c r="N4" s="7" t="n">
+      <c r="O4" s="6" t="n">
         <v>8124</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="P4" s="6" t="n"/>
+      <c r="Q4" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="R4" s="6" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="S4" s="7" t="n">
         <v>2166.44</v>
       </c>
-      <c r="P4" s="6" t="n">
+      <c r="T4" s="7" t="n">
         <v>2314.04</v>
       </c>
-      <c r="Q4" s="6" t="n">
+      <c r="U4" s="7" t="n">
         <v>46.28</v>
       </c>
-      <c r="R4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="6" t="n">
+      <c r="V4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="7" t="n">
         <v>2360.32</v>
       </c>
-      <c r="Y4" s="4" t="inlineStr">
+      <c r="AC4" s="4" t="inlineStr">
         <is>
           <t>Überfakturierung</t>
         </is>
@@ -828,45 +862,57 @@
         </is>
       </c>
       <c r="L5" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M5" s="11" t="n">
         <v>26.42</v>
       </c>
-      <c r="M5" s="10" t="n">
+      <c r="N5" s="11" t="n">
         <v>20.82145196945338</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="O5" s="10" t="n">
         <v>9952</v>
       </c>
-      <c r="O5" s="10" t="n">
+      <c r="P5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="10" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="S5" s="11" t="n">
         <v>2642</v>
       </c>
-      <c r="P5" s="10" t="n">
+      <c r="T5" s="11" t="n">
         <v>2072.1509</v>
       </c>
-      <c r="Q5" s="10" t="n">
+      <c r="U5" s="11" t="n">
         <v>41.443</v>
       </c>
-      <c r="R5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="10" t="n">
+      <c r="V5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="11" t="n">
         <v>2113.5939</v>
       </c>
-      <c r="Y5" s="8" t="inlineStr">
+      <c r="AC5" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -927,45 +973,57 @@
         </is>
       </c>
       <c r="L6" s="6" t="n">
+        <v>6500</v>
+      </c>
+      <c r="M6" s="7" t="n">
         <v>28.22</v>
       </c>
-      <c r="M6" s="6" t="n">
+      <c r="N6" s="7" t="n">
         <v>27.82761283077139</v>
       </c>
-      <c r="N6" s="7" t="n">
+      <c r="O6" s="6" t="n">
         <v>6411.15</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="P6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="S6" s="7" t="n">
         <v>1834.3</v>
       </c>
-      <c r="P6" s="6" t="n">
+      <c r="T6" s="7" t="n">
         <v>1784.07</v>
       </c>
-      <c r="Q6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="6" t="n">
+      <c r="U6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="7" t="n">
         <v>1784.07</v>
       </c>
-      <c r="Y6" s="4" t="inlineStr">
+      <c r="AC6" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1026,45 +1084,57 @@
         </is>
       </c>
       <c r="L7" s="10" t="n">
+        <v>6300</v>
+      </c>
+      <c r="M7" s="11" t="n">
         <v>28.22</v>
       </c>
-      <c r="M7" s="10" t="n">
+      <c r="N7" s="11" t="n">
         <v>28.7567051333068</v>
       </c>
-      <c r="N7" s="11" t="n">
+      <c r="O7" s="10" t="n">
         <v>6282.5</v>
       </c>
-      <c r="O7" s="10" t="n">
+      <c r="P7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="10" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="S7" s="11" t="n">
         <v>1777.86</v>
       </c>
-      <c r="P7" s="10" t="n">
+      <c r="T7" s="11" t="n">
         <v>1806.64</v>
       </c>
-      <c r="Q7" s="10" t="n">
+      <c r="U7" s="11" t="n">
         <v>35.56</v>
       </c>
-      <c r="R7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="10" t="n">
+      <c r="V7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="11" t="n">
         <v>1842.2</v>
       </c>
-      <c r="Y7" s="8" t="inlineStr">
+      <c r="AC7" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1125,45 +1195,57 @@
         </is>
       </c>
       <c r="L8" s="10" t="n">
+        <v>4200</v>
+      </c>
+      <c r="M8" s="11" t="n">
         <v>30.02</v>
       </c>
-      <c r="M8" s="10" t="n">
+      <c r="N8" s="11" t="n">
         <v>30.07011686143573</v>
       </c>
-      <c r="N8" s="11" t="n">
+      <c r="O8" s="10" t="n">
         <v>4193</v>
       </c>
-      <c r="O8" s="10" t="n">
+      <c r="P8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="10" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="S8" s="11" t="n">
         <v>1260.84</v>
       </c>
-      <c r="P8" s="10" t="n">
+      <c r="T8" s="11" t="n">
         <v>1260.84</v>
       </c>
-      <c r="Q8" s="10" t="n">
+      <c r="U8" s="11" t="n">
         <v>37.83</v>
       </c>
-      <c r="R8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="10" t="n">
+      <c r="V8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="11" t="n">
         <v>1298.67</v>
       </c>
-      <c r="Y8" s="8" t="inlineStr">
+      <c r="AC8" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1231,45 +1313,55 @@
         </is>
       </c>
       <c r="L11" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="M11" s="7" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="N11" s="7" t="n">
         <v>67.50464396284829</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="O11" s="6" t="n">
         <v>323</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="P11" s="6" t="n"/>
+      <c r="Q11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="S11" s="7" t="n">
         <v>235.72</v>
       </c>
-      <c r="P11" s="6" t="n">
+      <c r="T11" s="7" t="n">
         <v>218.04</v>
       </c>
-      <c r="Q11" s="6" t="n">
+      <c r="U11" s="7" t="n">
         <v>3.27</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" s="6" t="n">
+      <c r="V11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="7" t="n">
         <v>221.31</v>
       </c>
-      <c r="Y11" s="4" t="inlineStr">
+      <c r="AC11" s="4" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1330,45 +1422,57 @@
         </is>
       </c>
       <c r="L12" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="M12" s="11" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="M12" s="10" t="n">
+      <c r="N12" s="11" t="n">
         <v>19.99253205128205</v>
       </c>
-      <c r="N12" s="11" t="n">
+      <c r="O12" s="10" t="n">
         <v>312</v>
       </c>
-      <c r="O12" s="10" t="n">
+      <c r="P12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="10" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S12" s="11" t="n">
         <v>235.72</v>
       </c>
-      <c r="P12" s="10" t="n">
+      <c r="T12" s="11" t="n">
         <v>62.3767</v>
       </c>
-      <c r="Q12" s="10" t="n">
+      <c r="U12" s="11" t="n">
         <v>1.2476</v>
       </c>
-      <c r="R12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" s="10" t="n">
+      <c r="V12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="11" t="n">
         <v>63.6243</v>
       </c>
-      <c r="Y12" s="8" t="inlineStr">
+      <c r="AC12" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1429,45 +1533,57 @@
         </is>
       </c>
       <c r="L13" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="M13" s="11" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="M13" s="10" t="n">
+      <c r="N13" s="11" t="n">
         <v>26.22824207492796</v>
       </c>
-      <c r="N13" s="11" t="n">
+      <c r="O13" s="10" t="n">
         <v>347</v>
       </c>
-      <c r="O13" s="10" t="n">
+      <c r="P13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="10" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="S13" s="11" t="n">
         <v>235.72</v>
       </c>
-      <c r="P13" s="10" t="n">
+      <c r="T13" s="11" t="n">
         <v>91.012</v>
       </c>
-      <c r="Q13" s="10" t="n">
+      <c r="U13" s="11" t="n">
         <v>1.8201</v>
       </c>
-      <c r="R13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X13" s="10" t="n">
+      <c r="V13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="11" t="n">
         <v>92.8321</v>
       </c>
-      <c r="Y13" s="8" t="inlineStr">
+      <c r="AC13" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1528,45 +1644,57 @@
         </is>
       </c>
       <c r="L14" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="M14" s="11" t="n">
         <v>58.92999999999999</v>
       </c>
-      <c r="M14" s="10" t="n">
+      <c r="N14" s="11" t="n">
         <v>26.50052104208416</v>
       </c>
-      <c r="N14" s="11" t="n">
+      <c r="O14" s="10" t="n">
         <v>499</v>
       </c>
-      <c r="O14" s="10" t="n">
+      <c r="P14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="10" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="S14" s="11" t="n">
         <v>294.65</v>
       </c>
-      <c r="P14" s="10" t="n">
+      <c r="T14" s="11" t="n">
         <v>132.2376</v>
       </c>
-      <c r="Q14" s="10" t="n">
+      <c r="U14" s="11" t="n">
         <v>2.6454</v>
       </c>
-      <c r="R14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" s="10" t="n">
+      <c r="V14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="11" t="n">
         <v>134.883</v>
       </c>
-      <c r="Y14" s="8" t="inlineStr">
+      <c r="AC14" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1627,45 +1755,57 @@
         </is>
       </c>
       <c r="L15" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="M15" s="7" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="N15" s="7" t="n">
         <v>26.50053459119497</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="O15" s="6" t="n">
         <v>318</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="P15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="S15" s="7" t="n">
         <v>235.72</v>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="T15" s="7" t="n">
         <v>84.2717</v>
       </c>
-      <c r="Q15" s="6" t="n">
+      <c r="U15" s="7" t="n">
         <v>1.6859</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" s="6" t="n">
+      <c r="V15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="7" t="n">
         <v>85.9576</v>
       </c>
-      <c r="Y15" s="4" t="inlineStr">
+      <c r="AC15" s="4" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1726,45 +1866,57 @@
         </is>
       </c>
       <c r="L16" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="M16" s="11" t="n">
         <v>58.92999999999999</v>
       </c>
-      <c r="M16" s="10" t="n">
+      <c r="N16" s="11" t="n">
         <v>27.35258517034068</v>
       </c>
-      <c r="N16" s="11" t="n">
+      <c r="O16" s="10" t="n">
         <v>499</v>
       </c>
-      <c r="O16" s="10" t="n">
+      <c r="P16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="10" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="S16" s="11" t="n">
         <v>294.65</v>
       </c>
-      <c r="P16" s="10" t="n">
+      <c r="T16" s="11" t="n">
         <v>136.4894</v>
       </c>
-      <c r="Q16" s="10" t="n">
+      <c r="U16" s="11" t="n">
         <v>2.7292</v>
       </c>
-      <c r="R16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" s="10" t="n">
+      <c r="V16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="11" t="n">
         <v>139.2186</v>
       </c>
-      <c r="Y16" s="8" t="inlineStr">
+      <c r="AC16" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1832,45 +1984,55 @@
         </is>
       </c>
       <c r="L19" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M19" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="M19" s="6" t="n">
+      <c r="N19" s="7" t="n">
         <v>214.52</v>
       </c>
-      <c r="N19" s="7" t="n">
+      <c r="O19" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="O19" s="6" t="n">
+      <c r="P19" s="6" t="n"/>
+      <c r="Q19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="S19" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="P19" s="6" t="n">
+      <c r="T19" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="Q19" s="6" t="n">
+      <c r="U19" s="7" t="n">
         <v>2.15</v>
       </c>
-      <c r="R19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X19" s="6" t="n">
+      <c r="V19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="7" t="n">
         <v>55.78</v>
       </c>
-      <c r="Y19" s="4" t="inlineStr">
+      <c r="AC19" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1931,45 +2093,57 @@
         </is>
       </c>
       <c r="L20" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="M20" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="M20" s="10" t="n">
+      <c r="N20" s="11" t="n">
         <v>84.53708191953466</v>
       </c>
-      <c r="N20" s="11" t="n">
+      <c r="O20" s="10" t="n">
         <v>61.89</v>
       </c>
-      <c r="O20" s="10" t="n">
+      <c r="P20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="P20" s="10" t="n">
+      <c r="T20" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="Q20" s="10" t="n">
+      <c r="U20" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="R20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" s="10" t="n">
+      <c r="V20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="Y20" s="8" t="inlineStr">
+      <c r="AC20" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2030,45 +2204,57 @@
         </is>
       </c>
       <c r="L21" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="M21" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="M21" s="10" t="n">
+      <c r="N21" s="11" t="n">
         <v>118.4514376273489</v>
       </c>
-      <c r="N21" s="11" t="n">
+      <c r="O21" s="10" t="n">
         <v>44.17</v>
       </c>
-      <c r="O21" s="10" t="n">
+      <c r="P21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="10" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="S21" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="P21" s="10" t="n">
+      <c r="T21" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="Q21" s="10" t="n">
+      <c r="U21" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="R21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X21" s="10" t="n">
+      <c r="V21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="Y21" s="8" t="inlineStr">
+      <c r="AC21" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2129,45 +2315,57 @@
         </is>
       </c>
       <c r="L22" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M22" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="M22" s="6" t="n">
+      <c r="N22" s="7" t="n">
         <v>74.12344827586207</v>
       </c>
-      <c r="N22" s="7" t="n">
+      <c r="O22" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="O22" s="6" t="n">
+      <c r="P22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="P22" s="6" t="n">
+      <c r="T22" s="7" t="n">
         <v>21.4958</v>
       </c>
-      <c r="Q22" s="6" t="n">
+      <c r="U22" s="7" t="n">
         <v>0.4304</v>
       </c>
-      <c r="R22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X22" s="6" t="n">
+      <c r="V22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="7" t="n">
         <v>21.9262</v>
       </c>
-      <c r="Y22" s="4" t="inlineStr">
+      <c r="AC22" s="4" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -2228,45 +2426,57 @@
         </is>
       </c>
       <c r="L23" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="M23" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="M23" s="10" t="n">
+      <c r="N23" s="11" t="n">
         <v>61.55294117647059</v>
       </c>
-      <c r="N23" s="11" t="n">
+      <c r="O23" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="O23" s="10" t="n">
+      <c r="P23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="P23" s="10" t="n">
+      <c r="T23" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="Q23" s="10" t="n">
+      <c r="U23" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="R23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X23" s="10" t="n">
+      <c r="V23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="Y23" s="8" t="inlineStr">
+      <c r="AC23" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2327,45 +2537,57 @@
         </is>
       </c>
       <c r="L24" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="M24" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="M24" s="10" t="n">
+      <c r="N24" s="11" t="n">
         <v>55.07368421052632</v>
       </c>
-      <c r="N24" s="11" t="n">
+      <c r="O24" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="O24" s="10" t="n">
+      <c r="P24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="10" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="S24" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="P24" s="10" t="n">
+      <c r="T24" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="Q24" s="10" t="n">
+      <c r="U24" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="R24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" s="10" t="n">
+      <c r="V24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="Y24" s="8" t="inlineStr">
+      <c r="AC24" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2432,42 +2654,52 @@
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L27" s="6" t="n"/>
-      <c r="M27" s="6" t="n">
+      <c r="L27" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="7" t="n">
         <v>378</v>
       </c>
-      <c r="N27" s="7" t="n">
+      <c r="O27" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="O27" s="6" t="n"/>
-      <c r="P27" s="6" t="n">
+      <c r="P27" s="6" t="n"/>
+      <c r="Q27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="S27" s="7" t="n"/>
+      <c r="T27" s="7" t="n">
         <v>75.59999999999999</v>
       </c>
-      <c r="Q27" s="6" t="n">
+      <c r="U27" s="7" t="n">
         <v>1.51</v>
       </c>
-      <c r="R27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X27" s="6" t="n">
+      <c r="V27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="7" t="n">
         <v>77.11</v>
       </c>
-      <c r="Y27" s="4" t="inlineStr">
+      <c r="AC27" s="4" t="inlineStr">
         <is>
           <t>Soll n/a</t>
         </is>
@@ -2527,42 +2759,54 @@
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L28" s="10" t="n"/>
-      <c r="M28" s="10" t="n">
+      <c r="L28" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="M28" s="11" t="n"/>
+      <c r="N28" s="11" t="n">
         <v>48.51057747284163</v>
       </c>
-      <c r="N28" s="11" t="n">
+      <c r="O28" s="10" t="n">
         <v>34.98</v>
       </c>
-      <c r="O28" s="10" t="n"/>
       <c r="P28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="10" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="S28" s="11" t="n"/>
+      <c r="T28" s="11" t="n">
         <v>16.969</v>
       </c>
-      <c r="Q28" s="10" t="n">
+      <c r="U28" s="11" t="n">
         <v>0.3395</v>
       </c>
-      <c r="R28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X28" s="10" t="n">
+      <c r="V28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="11" t="n">
         <v>17.3085</v>
       </c>
-      <c r="Y28" s="8" t="inlineStr">
+      <c r="AC28" s="8" t="inlineStr">
         <is>
           <t>Soll n/a</t>
         </is>
@@ -2622,42 +2866,54 @@
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L29" s="6" t="n"/>
-      <c r="M29" s="6" t="n">
+      <c r="L29" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="M29" s="7" t="n"/>
+      <c r="N29" s="7" t="n">
         <v>57.75849289684991</v>
       </c>
-      <c r="N29" s="7" t="n">
+      <c r="O29" s="6" t="n">
         <v>32.38</v>
       </c>
-      <c r="O29" s="6" t="n"/>
       <c r="P29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="S29" s="7" t="n"/>
+      <c r="T29" s="7" t="n">
         <v>18.7022</v>
       </c>
-      <c r="Q29" s="6" t="n">
+      <c r="U29" s="7" t="n">
         <v>0.3746</v>
       </c>
-      <c r="R29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X29" s="6" t="n">
+      <c r="V29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="7" t="n">
         <v>19.0768</v>
       </c>
-      <c r="Y29" s="4" t="inlineStr">
+      <c r="AC29" s="4" t="inlineStr">
         <is>
           <t>Soll n/a</t>
         </is>
@@ -2665,11 +2921,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A10:Y10"/>
-    <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="A3:Y3"/>
-    <mergeCell ref="A18:Y18"/>
-    <mergeCell ref="A26:Y26"/>
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A18:AC18"/>
+    <mergeCell ref="A3:AC3"/>
+    <mergeCell ref="A26:AC26"/>
+    <mergeCell ref="A10:AC10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Master-Nr/Sub-Nr transparency columns to all 4 billing reports
New columns (33 total, was 29):
- Col 3 Master-Nr: master shipment number (for subs) or own Auftragsnr (for masters)
- Col 4 Sub-Nr(n): comma-separated list of all sub-order numbers
- Col 5 Anzahl Subs: count of consolidated sub-shipments
- Col 6 Ist Master: 'Ja' if row is the consolidated master

Consolidation logic (POST only — PRE has no master/sub):
- Sub rows removed from output (not shown separately)
- Sub financials (AX Fracht, Diesel, Maut, etc.) summed into master row
- Master's physical dimensions (Tonnage/Stellplätze) preserved as-is
- Cluster stats recomputed on consolidated data only

Impact: GEZE 1191 sub-rows removed, Helu 94 sub-rows removed.

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/geze_dinas_vergleich.xlsx
+++ b/output/billing_report/geze_dinas_vergleich.xlsx
@@ -117,11 +117,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -129,11 +129,11 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -503,44 +503,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC29"/>
+  <dimension ref="A1:AG28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
     <col width="9" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
-    <col width="9" customWidth="1" min="23" max="23"/>
-    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
     <col width="9" customWidth="1" min="25" max="25"/>
     <col width="9" customWidth="1" min="26" max="26"/>
     <col width="9" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="9" customWidth="1" min="28" max="28"/>
+    <col width="9" customWidth="1" min="29" max="29"/>
+    <col width="9" customWidth="1" min="30" max="30"/>
+    <col width="9" customWidth="1" min="31" max="31"/>
+    <col width="11" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GEZE GmbH (406035) — Dinas PRE vs AX POST  |  Cluster: 6  |  Sigma Verlust: -4,143 EUR</t>
+          <t>GEZE GmbH (406035) — Dinas PRE vs AX POST  |  Cluster: 6  |  Sigma Verlust: -3,567 EUR</t>
         </is>
       </c>
     </row>
@@ -557,135 +561,155 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Master-Nr</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Sub-Nr(n)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Anzahl Subs</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ist Master</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>Rech.-Nr</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Sendungsdatum</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Kunde</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Empf.PLZ</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Vers.PLZ</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Gew.band</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Basis Menge</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Basispreis</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Eff. Preis</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Tonnage kg</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Stellplätze</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Lademeter</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Volumen</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>Soll EUR</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Fracht EUR</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Diesel EUR</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Maut EUR</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Lademittel</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Peak EUR</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>Neben EUR</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr">
         <is>
           <t>EUST Zoll</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>Versich.</t>
         </is>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>Erlöse</t>
         </is>
       </c>
-      <c r="AC2" s="2" t="inlineStr">
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>Abw. Grund</t>
         </is>
@@ -694,7 +718,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>▶ 406035|71|FR|59|ueber 3000kg|EUR/100kg     n_PRE=1  n_POST=4  Ø Dinas=2,360.32 EUR  Ø AX=1,759.63 EUR  Δ=-600.69 EUR (-25.4%)  est.Verlust=-2,403 EUR  |  Eff. Dinas=28.48 | Eff. AX=26.87 | DLV=2,166.44 | ΔEff=-5.7%</t>
+          <t>▶ 406035|71|FR|59|ueber 3000kg|EUR/100kg     n_PRE=1  n_POST=3  Ø Dinas=2,360.32 EUR  Ø AX=1,751.49 EUR  Δ=-608.83 EUR (-25.8%)  est.Verlust=-1,826 EUR  |  Eff. Dinas=28.48 | Eff. AX=26.55 | DLV=2,166.44 | ΔEff=-6.8%</t>
         </is>
       </c>
     </row>
@@ -709,89 +733,83 @@
           <t>32901136</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>3769532</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>45812</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">59273    </t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">71229    </t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>ueber 3000kg</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="P4" s="5" t="n">
         <v>8200</v>
       </c>
-      <c r="M4" s="7" t="n">
+      <c r="Q4" s="7" t="n">
         <v>26.41999999999999</v>
       </c>
-      <c r="N4" s="7" t="n">
+      <c r="R4" s="7" t="n">
         <v>28.48399803052683</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="S4" s="5" t="n">
         <v>8124</v>
       </c>
-      <c r="P4" s="6" t="n"/>
-      <c r="Q4" s="6" t="n">
+      <c r="T4" s="5" t="n"/>
+      <c r="U4" s="5" t="n">
         <v>4.4</v>
       </c>
-      <c r="R4" s="6" t="n">
+      <c r="V4" s="5" t="n">
         <v>15.4</v>
       </c>
-      <c r="S4" s="7" t="n">
+      <c r="W4" s="7" t="n">
         <v>2166.44</v>
       </c>
-      <c r="T4" s="7" t="n">
+      <c r="X4" s="7" t="n">
         <v>2314.04</v>
       </c>
-      <c r="U4" s="7" t="n">
+      <c r="Y4" s="7" t="n">
         <v>46.28</v>
       </c>
-      <c r="V4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="Z4" s="7" t="n">
         <v>0</v>
       </c>
@@ -799,231 +817,255 @@
         <v>0</v>
       </c>
       <c r="AB4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="7" t="n">
         <v>2360.32</v>
       </c>
-      <c r="AC4" s="4" t="inlineStr">
+      <c r="AG4" s="4" t="inlineStr">
         <is>
           <t>Überfakturierung</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>7091200281042008</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>4251011138</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="H5" s="6" t="n">
         <v>45952</v>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>59273</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>ueber 3000kg</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L5" s="10" t="n">
+      <c r="P5" s="5" t="n">
         <v>10000</v>
       </c>
-      <c r="M5" s="11" t="n">
+      <c r="Q5" s="7" t="n">
         <v>26.42</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="R5" s="7" t="n">
         <v>20.82145196945338</v>
       </c>
-      <c r="O5" s="10" t="n">
+      <c r="S5" s="5" t="n">
         <v>9952</v>
       </c>
-      <c r="P5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="10" t="n">
+      <c r="T5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="5" t="n">
         <v>19.4</v>
       </c>
-      <c r="S5" s="11" t="n">
+      <c r="W5" s="7" t="n">
         <v>2642</v>
       </c>
-      <c r="T5" s="11" t="n">
+      <c r="X5" s="7" t="n">
         <v>2072.1509</v>
       </c>
-      <c r="U5" s="11" t="n">
+      <c r="Y5" s="7" t="n">
         <v>41.443</v>
       </c>
-      <c r="V5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="11" t="n">
+      <c r="Z5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="7" t="n">
         <v>2113.5939</v>
       </c>
-      <c r="AC5" s="8" t="inlineStr">
+      <c r="AG5" s="4" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>7091200282378007</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>2573273</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>45982</v>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>7091200283310006</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="8" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>2577017</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>46006</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>59273</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>ueber 3000kg</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L6" s="6" t="n">
-        <v>6500</v>
-      </c>
-      <c r="M6" s="7" t="n">
+      <c r="P6" s="9" t="n">
+        <v>6300</v>
+      </c>
+      <c r="Q6" s="11" t="n">
         <v>28.22</v>
       </c>
-      <c r="N6" s="7" t="n">
-        <v>27.82761283077139</v>
-      </c>
-      <c r="O6" s="6" t="n">
-        <v>6411.15</v>
-      </c>
-      <c r="P6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="6" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="S6" s="7" t="n">
-        <v>1834.3</v>
-      </c>
-      <c r="T6" s="7" t="n">
-        <v>1784.07</v>
-      </c>
-      <c r="U6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="7" t="n">
-        <v>1784.07</v>
-      </c>
-      <c r="AC6" s="4" t="inlineStr">
+      <c r="R6" s="11" t="n">
+        <v>28.7567051333068</v>
+      </c>
+      <c r="S6" s="9" t="n">
+        <v>6282.5</v>
+      </c>
+      <c r="T6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="9" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="W6" s="11" t="n">
+        <v>1777.86</v>
+      </c>
+      <c r="X6" s="11" t="n">
+        <v>1806.64</v>
+      </c>
+      <c r="Y6" s="11" t="n">
+        <v>35.56</v>
+      </c>
+      <c r="Z6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="11" t="n">
+        <v>1842.2</v>
+      </c>
+      <c r="AG6" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1037,93 +1079,87 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>7091200283310006</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>2577017</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>46006</v>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
+          <t>7091200283963004</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>2582348</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>46036</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>59273</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="L7" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>ueber 3000kg</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="O7" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L7" s="10" t="n">
-        <v>6300</v>
-      </c>
-      <c r="M7" s="11" t="n">
-        <v>28.22</v>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v>28.7567051333068</v>
-      </c>
-      <c r="O7" s="10" t="n">
-        <v>6282.5</v>
-      </c>
-      <c r="P7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="10" t="n">
-        <v>12.85</v>
-      </c>
-      <c r="S7" s="11" t="n">
-        <v>1777.86</v>
-      </c>
-      <c r="T7" s="11" t="n">
-        <v>1806.64</v>
-      </c>
-      <c r="U7" s="11" t="n">
-        <v>35.56</v>
-      </c>
-      <c r="V7" s="11" t="n">
-        <v>0</v>
+      <c r="P7" s="9" t="n">
+        <v>4200</v>
+      </c>
+      <c r="Q7" s="11" t="n">
+        <v>30.02</v>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>30.07011686143573</v>
+      </c>
+      <c r="S7" s="9" t="n">
+        <v>4193</v>
+      </c>
+      <c r="T7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="9" t="n">
+        <v>6.61</v>
       </c>
       <c r="W7" s="11" t="n">
-        <v>0</v>
+        <v>1260.84</v>
       </c>
       <c r="X7" s="11" t="n">
-        <v>0</v>
+        <v>1260.84</v>
       </c>
       <c r="Y7" s="11" t="n">
-        <v>0</v>
+        <v>37.83</v>
       </c>
       <c r="Z7" s="11" t="n">
         <v>0</v>
@@ -1132,236 +1168,260 @@
         <v>0</v>
       </c>
       <c r="AB7" s="11" t="n">
-        <v>1842.2</v>
-      </c>
-      <c r="AC7" s="8" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="11" t="n">
+        <v>1298.67</v>
+      </c>
+      <c r="AG7" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>▶ 406035|71|FR|77|bis 500kg|EUR/100kg     n_PRE=1  n_POST=12  Ø Dinas=221.31 EUR  Ø AX=120.36 EUR  Δ=-100.95 EUR (-45.6%)  est.Verlust=-1,211 EUR  |  Eff. Dinas=67.50 | Eff. AX=29.47 | DLV=235.72 | ΔEff=-56.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>alt</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>32925122</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>3773387</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>45849</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>GEZE GmbH</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77164    </t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71229    </t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>bis 500kg</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>EUR/100kg</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>58.93000000000001</v>
+      </c>
+      <c r="R10" s="7" t="n">
+        <v>67.50464396284829</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>323</v>
+      </c>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="5" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="W10" s="7" t="n">
+        <v>235.72</v>
+      </c>
+      <c r="X10" s="7" t="n">
+        <v>218.04</v>
+      </c>
+      <c r="Y10" s="7" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="Z10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="7" t="n">
+        <v>221.31</v>
+      </c>
+      <c r="AG10" s="4" t="inlineStr">
+        <is>
+          <t>Unterfakturierung</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>7091200283963004</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>2582348</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>46036</v>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>7091200282105009</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>2568656</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>45975</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>59273</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>77170</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>ueber 3000kg</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>bis 500kg</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L8" s="10" t="n">
-        <v>4200</v>
-      </c>
-      <c r="M8" s="11" t="n">
-        <v>30.02</v>
-      </c>
-      <c r="N8" s="11" t="n">
-        <v>30.07011686143573</v>
-      </c>
-      <c r="O8" s="10" t="n">
-        <v>4193</v>
-      </c>
-      <c r="P8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="10" t="n">
-        <v>6.61</v>
-      </c>
-      <c r="S8" s="11" t="n">
-        <v>1260.84</v>
-      </c>
-      <c r="T8" s="11" t="n">
-        <v>1260.84</v>
-      </c>
-      <c r="U8" s="11" t="n">
-        <v>37.83</v>
-      </c>
-      <c r="V8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="11" t="n">
-        <v>1298.67</v>
-      </c>
-      <c r="AC8" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>▶ 406035|71|FR|77|bis 500kg|EUR/100kg     n_PRE=1  n_POST=12  Ø Dinas=221.31 EUR  Ø AX=120.36 EUR  Δ=-100.95 EUR (-45.6%)  est.Verlust=-1,211 EUR  |  Eff. Dinas=67.50 | Eff. AX=29.47 | DLV=235.72 | ΔEff=-56.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>alt</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>32925122</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>3773387</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>45849</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>GEZE GmbH</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">77164    </t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71229    </t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>bis 500kg</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>EUR/100kg</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="n">
+      <c r="P11" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="M11" s="7" t="n">
+      <c r="Q11" s="11" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="N11" s="7" t="n">
-        <v>67.50464396284829</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>323</v>
-      </c>
-      <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="S11" s="7" t="n">
+      <c r="R11" s="11" t="n">
+        <v>19.99253205128205</v>
+      </c>
+      <c r="S11" s="9" t="n">
+        <v>312</v>
+      </c>
+      <c r="T11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="W11" s="11" t="n">
         <v>235.72</v>
       </c>
-      <c r="T11" s="7" t="n">
-        <v>218.04</v>
-      </c>
-      <c r="U11" s="7" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="V11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="7" t="n">
-        <v>221.31</v>
-      </c>
-      <c r="AC11" s="4" t="inlineStr">
+      <c r="X11" s="11" t="n">
+        <v>62.3767</v>
+      </c>
+      <c r="Y11" s="11" t="n">
+        <v>1.2476</v>
+      </c>
+      <c r="Z11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" s="11" t="n">
+        <v>63.6243</v>
+      </c>
+      <c r="AG11" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1375,93 +1435,87 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>7091200282105009</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>2568656</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>45975</v>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+          <t>7091200282730003</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>2573273</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>45989</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>77170</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>bis 500kg</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K12" s="8" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L12" s="10" t="n">
+      <c r="P12" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="M12" s="11" t="n">
+      <c r="Q12" s="11" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="N12" s="11" t="n">
-        <v>19.99253205128205</v>
-      </c>
-      <c r="O12" s="10" t="n">
-        <v>312</v>
-      </c>
-      <c r="P12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="S12" s="11" t="n">
+      <c r="R12" s="11" t="n">
+        <v>26.22824207492796</v>
+      </c>
+      <c r="S12" s="9" t="n">
+        <v>347</v>
+      </c>
+      <c r="T12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="9" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="W12" s="11" t="n">
         <v>235.72</v>
       </c>
-      <c r="T12" s="11" t="n">
-        <v>62.3767</v>
-      </c>
-      <c r="U12" s="11" t="n">
-        <v>1.2476</v>
-      </c>
-      <c r="V12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W12" s="11" t="n">
-        <v>0</v>
-      </c>
       <c r="X12" s="11" t="n">
-        <v>0</v>
+        <v>91.012</v>
       </c>
       <c r="Y12" s="11" t="n">
-        <v>0</v>
+        <v>1.8201</v>
       </c>
       <c r="Z12" s="11" t="n">
         <v>0</v>
@@ -1470,9 +1524,21 @@
         <v>0</v>
       </c>
       <c r="AB12" s="11" t="n">
-        <v>63.6243</v>
-      </c>
-      <c r="AC12" s="8" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="11" t="n">
+        <v>92.8321</v>
+      </c>
+      <c r="AG12" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
@@ -1486,553 +1552,583 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>7091200282730003</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>2573273</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>45989</v>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+          <t>7091200283078005</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="8" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>2577017</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>45996</v>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>77170</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t>bis 500kg</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr">
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K13" s="8" t="inlineStr">
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L13" s="10" t="n">
+      <c r="P13" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="Q13" s="11" t="n">
+        <v>58.92999999999999</v>
+      </c>
+      <c r="R13" s="11" t="n">
+        <v>26.50052104208416</v>
+      </c>
+      <c r="S13" s="9" t="n">
+        <v>499</v>
+      </c>
+      <c r="T13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="9" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="W13" s="11" t="n">
+        <v>294.65</v>
+      </c>
+      <c r="X13" s="11" t="n">
+        <v>132.2376</v>
+      </c>
+      <c r="Y13" s="11" t="n">
+        <v>2.6454</v>
+      </c>
+      <c r="Z13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="11" t="n">
+        <v>134.883</v>
+      </c>
+      <c r="AG13" s="8" t="inlineStr">
+        <is>
+          <t>Unterfakturierung</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>7091200283092001</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>2577017</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>45996</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>GEZE GmbH</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>77170</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>71229</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>bis 500kg</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>EUR/100kg</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="M13" s="11" t="n">
+      <c r="Q14" s="7" t="n">
         <v>58.93000000000001</v>
       </c>
-      <c r="N13" s="11" t="n">
-        <v>26.22824207492796</v>
-      </c>
-      <c r="O13" s="10" t="n">
-        <v>347</v>
-      </c>
-      <c r="P13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="10" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="S13" s="11" t="n">
+      <c r="R14" s="7" t="n">
+        <v>26.50053459119497</v>
+      </c>
+      <c r="S14" s="5" t="n">
+        <v>318</v>
+      </c>
+      <c r="T14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="W14" s="7" t="n">
         <v>235.72</v>
       </c>
-      <c r="T13" s="11" t="n">
-        <v>91.012</v>
-      </c>
-      <c r="U13" s="11" t="n">
-        <v>1.8201</v>
-      </c>
-      <c r="V13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="11" t="n">
-        <v>92.8321</v>
-      </c>
-      <c r="AC13" s="8" t="inlineStr">
+      <c r="X14" s="7" t="n">
+        <v>84.2717</v>
+      </c>
+      <c r="Y14" s="7" t="n">
+        <v>1.6859</v>
+      </c>
+      <c r="Z14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" s="7" t="n">
+        <v>85.9576</v>
+      </c>
+      <c r="AG14" s="4" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>7091200283078005</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>2577017</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>45996</v>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>7091200283509004</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>2578458</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>46010</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>77170</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="L15" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>bis 500kg</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L14" s="10" t="n">
+      <c r="P15" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="M14" s="11" t="n">
+      <c r="Q15" s="11" t="n">
         <v>58.92999999999999</v>
       </c>
-      <c r="N14" s="11" t="n">
-        <v>26.50052104208416</v>
-      </c>
-      <c r="O14" s="10" t="n">
+      <c r="R15" s="11" t="n">
+        <v>27.35258517034068</v>
+      </c>
+      <c r="S15" s="9" t="n">
         <v>499</v>
       </c>
-      <c r="P14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="10" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="S14" s="11" t="n">
+      <c r="T15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="9" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="W15" s="11" t="n">
         <v>294.65</v>
       </c>
-      <c r="T14" s="11" t="n">
-        <v>132.2376</v>
-      </c>
-      <c r="U14" s="11" t="n">
-        <v>2.6454</v>
-      </c>
-      <c r="V14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="11" t="n">
-        <v>134.883</v>
-      </c>
-      <c r="AC14" s="8" t="inlineStr">
+      <c r="X15" s="11" t="n">
+        <v>136.4894</v>
+      </c>
+      <c r="Y15" s="11" t="n">
+        <v>2.7292</v>
+      </c>
+      <c r="Z15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="11" t="n">
+        <v>139.2186</v>
+      </c>
+      <c r="AG15" s="8" t="inlineStr">
         <is>
           <t>Unterfakturierung</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>▶ 406035|71|ES|08|bis 100kg|EUR/100kg     n_PRE=1  n_POST=52  Ø Dinas=55.78 EUR  Ø AX=48.01 EUR  Δ=-7.77 EUR (-13.9%)  est.Verlust=-404 EUR  |  Eff. Dinas=214.52 | Eff. AX=503.90 | DLV=53.63 | ΔEff=+134.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>alt</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>32883174</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>3761976</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>45770</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>GEZE GmbH</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08800    </t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71229    </t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>bis 100kg</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>EUR/100kg</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q18" s="7" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="R18" s="7" t="n">
+        <v>214.52</v>
+      </c>
+      <c r="S18" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="T18" s="5" t="n"/>
+      <c r="U18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="5" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="W18" s="7" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="X18" s="7" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="Y18" s="7" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="Z18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="7" t="n">
+        <v>55.78</v>
+      </c>
+      <c r="AG18" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>7091200283092001</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>2577017</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>45996</v>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>7091200280306002</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="8" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>2560101</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>45937</v>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>77170</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>08907</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>bis 500kg</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>bis 100kg</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="O19" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="M15" s="7" t="n">
-        <v>58.93000000000001</v>
-      </c>
-      <c r="N15" s="7" t="n">
-        <v>26.50053459119497</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>318</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="S15" s="7" t="n">
-        <v>235.72</v>
-      </c>
-      <c r="T15" s="7" t="n">
-        <v>84.2717</v>
-      </c>
-      <c r="U15" s="7" t="n">
-        <v>1.6859</v>
-      </c>
-      <c r="V15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="7" t="n">
-        <v>85.9576</v>
-      </c>
-      <c r="AC15" s="4" t="inlineStr">
-        <is>
-          <t>Unterfakturierung</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>7091200283509004</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>2578458</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>46010</v>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>GEZE GmbH</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>77170</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>71229</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>bis 500kg</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>EUR/100kg</t>
-        </is>
-      </c>
-      <c r="L16" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="M16" s="11" t="n">
-        <v>58.92999999999999</v>
-      </c>
-      <c r="N16" s="11" t="n">
-        <v>27.35258517034068</v>
-      </c>
-      <c r="O16" s="10" t="n">
-        <v>499</v>
-      </c>
-      <c r="P16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="10" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="S16" s="11" t="n">
-        <v>294.65</v>
-      </c>
-      <c r="T16" s="11" t="n">
-        <v>136.4894</v>
-      </c>
-      <c r="U16" s="11" t="n">
-        <v>2.7292</v>
-      </c>
-      <c r="V16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="11" t="n">
-        <v>139.2186</v>
-      </c>
-      <c r="AC16" s="8" t="inlineStr">
-        <is>
-          <t>Unterfakturierung</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>▶ 406035|71|ES|08|bis 100kg|EUR/100kg     n_PRE=1  n_POST=52  Ø Dinas=55.78 EUR  Ø AX=48.01 EUR  Δ=-7.77 EUR (-13.9%)  est.Verlust=-404 EUR  |  Eff. Dinas=214.52 | Eff. AX=503.90 | DLV=53.63 | ΔEff=+134.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>alt</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>32883174</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>3761976</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>45770</v>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>GEZE GmbH</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08800    </t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71229    </t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>bis 100kg</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>EUR/100kg</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="n">
+      <c r="P19" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M19" s="7" t="n">
+      <c r="Q19" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="N19" s="7" t="n">
-        <v>214.52</v>
-      </c>
-      <c r="O19" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="S19" s="7" t="n">
+      <c r="R19" s="11" t="n">
+        <v>84.53708191953466</v>
+      </c>
+      <c r="S19" s="9" t="n">
+        <v>61.89</v>
+      </c>
+      <c r="T19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="T19" s="7" t="n">
-        <v>53.63</v>
-      </c>
-      <c r="U19" s="7" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="V19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="7" t="n">
-        <v>55.78</v>
-      </c>
-      <c r="AC19" s="4" t="inlineStr">
+      <c r="X19" s="11" t="n">
+        <v>52.32</v>
+      </c>
+      <c r="Y19" s="11" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="Z19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="11" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="AG19" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -2046,94 +2142,88 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>7091200280306002</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
+          <t>7091200280411003</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>2560101</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="H20" s="10" t="n">
         <v>45937</v>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>08907</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>08205</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>bis 100kg</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="N20" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K20" s="8" t="inlineStr">
+      <c r="O20" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L20" s="10" t="n">
+      <c r="P20" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M20" s="11" t="n">
+      <c r="Q20" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="N20" s="11" t="n">
-        <v>84.53708191953466</v>
-      </c>
-      <c r="O20" s="10" t="n">
-        <v>61.89</v>
-      </c>
-      <c r="P20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="11" t="n">
+      <c r="R20" s="11" t="n">
+        <v>118.4514376273489</v>
+      </c>
+      <c r="S20" s="9" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="T20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="9" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="W20" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="T20" s="11" t="n">
+      <c r="X20" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="U20" s="11" t="n">
+      <c r="Y20" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="V20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="11" t="n">
-        <v>0</v>
-      </c>
       <c r="Z20" s="11" t="n">
         <v>0</v>
       </c>
@@ -2141,233 +2231,257 @@
         <v>0</v>
       </c>
       <c r="AB20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="AC20" s="8" t="inlineStr">
+      <c r="AG20" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>7091200280411003</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>7091200280558005</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>2560101</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
-        <v>45937</v>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="H21" s="6" t="n">
+        <v>45940</v>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>08205</t>
-        </is>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>08830</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I21" s="8" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>bis 100kg</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K21" s="8" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L21" s="10" t="n">
+      <c r="P21" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="M21" s="11" t="n">
+      <c r="Q21" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="N21" s="11" t="n">
-        <v>118.4514376273489</v>
-      </c>
-      <c r="O21" s="10" t="n">
-        <v>44.17</v>
-      </c>
-      <c r="P21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="10" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="S21" s="11" t="n">
+      <c r="R21" s="7" t="n">
+        <v>74.12344827586207</v>
+      </c>
+      <c r="S21" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="T21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" s="7" t="n">
         <v>53.63</v>
       </c>
-      <c r="T21" s="11" t="n">
+      <c r="X21" s="7" t="n">
+        <v>21.4958</v>
+      </c>
+      <c r="Y21" s="7" t="n">
+        <v>0.4304</v>
+      </c>
+      <c r="Z21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="7" t="n">
+        <v>21.9262</v>
+      </c>
+      <c r="AG21" s="4" t="inlineStr">
+        <is>
+          <t>Unterfakturierung</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>7091200280444001</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>2560101</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>45940</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>GEZE GmbH</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>08830</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>71229</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>bis 100kg</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="inlineStr">
+        <is>
+          <t>EUR/100kg</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q22" s="11" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="R22" s="11" t="n">
+        <v>61.55294117647059</v>
+      </c>
+      <c r="S22" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="T22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" s="11" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="X22" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="U21" s="11" t="n">
+      <c r="Y22" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="V21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="11" t="n">
+      <c r="Z22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="AC21" s="8" t="inlineStr">
+      <c r="AG22" s="8" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>7091200280558005</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>2560101</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>45940</v>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>GEZE GmbH</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>08830</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>71229</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>bis 100kg</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>EUR/100kg</t>
-        </is>
-      </c>
-      <c r="L22" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="M22" s="7" t="n">
-        <v>53.63</v>
-      </c>
-      <c r="N22" s="7" t="n">
-        <v>74.12344827586207</v>
-      </c>
-      <c r="O22" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="P22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="7" t="n">
-        <v>53.63</v>
-      </c>
-      <c r="T22" s="7" t="n">
-        <v>21.4958</v>
-      </c>
-      <c r="U22" s="7" t="n">
-        <v>0.4304</v>
-      </c>
-      <c r="V22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="7" t="n">
-        <v>21.9262</v>
-      </c>
-      <c r="AC22" s="4" t="inlineStr">
-        <is>
-          <t>Unterfakturierung</t>
         </is>
       </c>
     </row>
@@ -2379,94 +2493,88 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>7091200280444001</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
+          <t>7091200280579000</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>2560101</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
-        <v>45940</v>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="H23" s="10" t="n">
+        <v>45943</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>08830</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>08908</t>
+        </is>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
+      <c r="M23" s="8" t="inlineStr">
         <is>
           <t>bis 100kg</t>
         </is>
       </c>
-      <c r="J23" s="8" t="inlineStr">
+      <c r="N23" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K23" s="8" t="inlineStr">
+      <c r="O23" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L23" s="10" t="n">
+      <c r="P23" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M23" s="11" t="n">
+      <c r="Q23" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="N23" s="11" t="n">
-        <v>61.55294117647059</v>
-      </c>
-      <c r="O23" s="10" t="n">
-        <v>85</v>
-      </c>
-      <c r="P23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="11" t="n">
+      <c r="R23" s="11" t="n">
+        <v>55.07368421052632</v>
+      </c>
+      <c r="S23" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="T23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="9" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="W23" s="11" t="n">
         <v>53.63</v>
       </c>
-      <c r="T23" s="11" t="n">
+      <c r="X23" s="11" t="n">
         <v>52.32</v>
       </c>
-      <c r="U23" s="11" t="n">
+      <c r="Y23" s="11" t="n">
         <v>1.05</v>
       </c>
-      <c r="V23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="11" t="n">
-        <v>0</v>
-      </c>
       <c r="Z23" s="11" t="n">
         <v>0</v>
       </c>
@@ -2474,446 +2582,365 @@
         <v>0</v>
       </c>
       <c r="AB23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="11" t="n">
         <v>53.37</v>
       </c>
-      <c r="AC23" s="8" t="inlineStr">
+      <c r="AG23" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>▶ 406035|71|GR|56|bis 100kg|EUR/100kg     n_PRE=1  n_POST=2  Ø Dinas=77.11 EUR  Ø AX=18.19 EUR  Δ=-58.92 EUR (-76.4%)  est.Verlust=-118 EUR  |  Eff. Dinas=378.00 | Eff. AX=53.13 | DLV=n/a | ΔEff=-85.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>alt</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>32910451</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>3769530</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>45821</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>GEZE GmbH</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56535    </t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71229    </t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>bis 100kg</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>EUR/100kg</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q26" s="7" t="n"/>
+      <c r="R26" s="7" t="n">
+        <v>378</v>
+      </c>
+      <c r="S26" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="T26" s="5" t="n"/>
+      <c r="U26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" s="5" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="W26" s="7" t="n"/>
+      <c r="X26" s="7" t="n">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="Y26" s="7" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="Z26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="7" t="n">
+        <v>77.11</v>
+      </c>
+      <c r="AG26" s="4" t="inlineStr">
+        <is>
+          <t>Soll n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>neu</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>7091200280579000</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>7091200280723007</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>2560101</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
-        <v>45943</v>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="H27" s="10" t="n">
+        <v>45946</v>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>08908</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>564 29</t>
+        </is>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
         <is>
           <t>71229</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
+      <c r="M27" s="8" t="inlineStr">
         <is>
           <t>bis 100kg</t>
         </is>
       </c>
-      <c r="J24" s="8" t="inlineStr">
+      <c r="N27" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K24" s="8" t="inlineStr">
+      <c r="O27" s="8" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L24" s="10" t="n">
+      <c r="P27" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="M24" s="11" t="n">
-        <v>53.63</v>
-      </c>
-      <c r="N24" s="11" t="n">
-        <v>55.07368421052632</v>
-      </c>
-      <c r="O24" s="10" t="n">
-        <v>95</v>
-      </c>
-      <c r="P24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="10" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="S24" s="11" t="n">
-        <v>53.63</v>
-      </c>
-      <c r="T24" s="11" t="n">
-        <v>52.32</v>
-      </c>
-      <c r="U24" s="11" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="V24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="11" t="n">
-        <v>53.37</v>
-      </c>
-      <c r="AC24" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>▶ 406035|71|GR|56|bis 100kg|EUR/100kg     n_PRE=1  n_POST=2  Ø Dinas=77.11 EUR  Ø AX=18.19 EUR  Δ=-58.92 EUR (-76.4%)  est.Verlust=-118 EUR  |  Eff. Dinas=378.00 | Eff. AX=53.13 | DLV=n/a | ΔEff=-85.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>alt</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>32910451</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>3769530</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>45821</v>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="Q27" s="11" t="n"/>
+      <c r="R27" s="11" t="n">
+        <v>48.51057747284163</v>
+      </c>
+      <c r="S27" s="9" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="T27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" s="9" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="W27" s="11" t="n"/>
+      <c r="X27" s="11" t="n">
+        <v>16.969</v>
+      </c>
+      <c r="Y27" s="11" t="n">
+        <v>0.3395</v>
+      </c>
+      <c r="Z27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="11" t="n">
+        <v>17.3085</v>
+      </c>
+      <c r="AG27" s="8" t="inlineStr">
+        <is>
+          <t>Soll n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>7091200282614006</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>2573273</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>45989</v>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>GEZE GmbH</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>GR</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">56535    </t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71229    </t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>564 29</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>71229</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>bis 100kg</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>EUR/100kg</t>
         </is>
       </c>
-      <c r="L27" s="6" t="n">
+      <c r="P28" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n">
-        <v>378</v>
-      </c>
-      <c r="O27" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="P27" s="6" t="n"/>
-      <c r="Q27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="6" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S27" s="7" t="n"/>
-      <c r="T27" s="7" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="U27" s="7" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="V27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB27" s="7" t="n">
-        <v>77.11</v>
-      </c>
-      <c r="AC27" s="4" t="inlineStr">
-        <is>
-          <t>Soll n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>7091200280723007</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>2560101</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="n">
-        <v>45946</v>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>GEZE GmbH</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>564 29</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>71229</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>bis 100kg</t>
-        </is>
-      </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="K28" s="8" t="inlineStr">
-        <is>
-          <t>EUR/100kg</t>
-        </is>
-      </c>
-      <c r="L28" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="M28" s="11" t="n"/>
-      <c r="N28" s="11" t="n">
-        <v>48.51057747284163</v>
-      </c>
-      <c r="O28" s="10" t="n">
-        <v>34.98</v>
-      </c>
-      <c r="P28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="10" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="S28" s="11" t="n"/>
-      <c r="T28" s="11" t="n">
-        <v>16.969</v>
-      </c>
-      <c r="U28" s="11" t="n">
-        <v>0.3395</v>
-      </c>
-      <c r="V28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB28" s="11" t="n">
-        <v>17.3085</v>
-      </c>
-      <c r="AC28" s="8" t="inlineStr">
-        <is>
-          <t>Soll n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>7091200282614006</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>2573273</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>45989</v>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>GEZE GmbH</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>564 29</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>71229</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>bis 100kg</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>EUR/100kg</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="M29" s="7" t="n"/>
-      <c r="N29" s="7" t="n">
+      <c r="Q28" s="7" t="n"/>
+      <c r="R28" s="7" t="n">
         <v>57.75849289684991</v>
       </c>
-      <c r="O29" s="6" t="n">
+      <c r="S28" s="5" t="n">
         <v>32.38</v>
       </c>
-      <c r="P29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="6" t="n">
+      <c r="T28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" s="5" t="n">
         <v>0.23</v>
       </c>
-      <c r="S29" s="7" t="n"/>
-      <c r="T29" s="7" t="n">
+      <c r="W28" s="7" t="n"/>
+      <c r="X28" s="7" t="n">
         <v>18.7022</v>
       </c>
-      <c r="U29" s="7" t="n">
+      <c r="Y28" s="7" t="n">
         <v>0.3746</v>
       </c>
-      <c r="V29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB29" s="7" t="n">
+      <c r="Z28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="7" t="n">
         <v>19.0768</v>
       </c>
-      <c r="AC29" s="4" t="inlineStr">
+      <c r="AG28" s="4" t="inlineStr">
         <is>
           <t>Soll n/a</t>
         </is>
@@ -2921,11 +2948,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:AC1"/>
-    <mergeCell ref="A18:AC18"/>
-    <mergeCell ref="A3:AC3"/>
-    <mergeCell ref="A26:AC26"/>
-    <mergeCell ref="A10:AC10"/>
+    <mergeCell ref="A1:AG1"/>
+    <mergeCell ref="A17:AG17"/>
+    <mergeCell ref="A9:AG9"/>
+    <mergeCell ref="A3:AG3"/>
+    <mergeCell ref="A25:AG25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>